<commit_message>
ajuste de erros de imagem e remoção de campos da planilha modelo
</commit_message>
<xml_diff>
--- a/Planilha_Modelo_Importacao_Pedido_Mega12.xlsx
+++ b/Planilha_Modelo_Importacao_Pedido_Mega12.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="196">
   <si>
     <t>REDE MEGA 12 • PLANILHA MODELO DE IMPORTAÇÃO DE PEDIDOS</t>
   </si>
@@ -25,10 +25,10 @@
     <t>ALS 10 BAZAR E BRINQUEDOS LTDA  •  ESTRUTURA INTELIGENTE ANTI-ERRO</t>
   </si>
   <si>
-    <t>Uso: Compras, Feiras e Fornecedores</t>
-  </si>
-  <si>
-    <t>ℹ️ INSTRUÇÕES: Preencha os Dados do Fornecedor, Condições e Produtos. As colunas verdes e cinzas contêm fórmulas automáticas de conferência.</t>
+    <t>Uso: Compras e Fornecedores</t>
+  </si>
+  <si>
+    <t>ℹ️ INSTRUÇÕES: Preencha os Dados do Fornecedor, Condições e Produtos. A coluna TOTAL PEÇAS calcula automaticamente (= QTD/CX × QTD CX).</t>
   </si>
   <si>
     <t>1. DADOS DA EMPRESA COMPRADORA (DESTINATÁRIO - MEGA 12):</t>
@@ -121,7 +121,7 @@
     <t>CIF</t>
   </si>
   <si>
-    <t>Cond. Pagamento:</t>
+    <t>Cond. Pag.:</t>
   </si>
   <si>
     <t>30/60/90 Dias</t>
@@ -178,21 +178,6 @@
     <t>PREÇO UNIT. (R$)</t>
   </si>
   <si>
-    <t>% IPI</t>
-  </si>
-  <si>
-    <t>VALOR IPI (R$)</t>
-  </si>
-  <si>
-    <t>VALOR TOTAL (R$)</t>
-  </si>
-  <si>
-    <t>PDV SUGERIDO (R$)</t>
-  </si>
-  <si>
-    <t>MARGEM BRUTA (%)</t>
-  </si>
-  <si>
     <t>652</t>
   </si>
   <si>
@@ -274,10 +259,7 @@
     <t>TOTAIS CONSOLIDADOS DO PEDIDO:</t>
   </si>
   <si>
-    <t>REGRAS MANDATÓRIAS DE RECEBIMENTO &amp; FATURAMENTO (REDE MEGA 12):</t>
-  </si>
-  <si>
-    <t>TOTAL GERAL DO PEDIDO (MERCADORIAS + IPI):</t>
+    <t>REGRAS MANDATÓRIAS DE RECEBIMENTO &amp; FATURAMENTO (REDE MEGA 12 - CD IRATI):</t>
   </si>
   <si>
     <t>1. Boletos NÃO devem exceder o valor de R$ 9.999,00 por título.</t>
@@ -466,15 +448,30 @@
     <t>Exemplos: 30/60/90 Dias, Boleto 30 Dias, À Vista. O sistema gera automaticamente o fluxo de duplicatas financeiras.</t>
   </si>
   <si>
+    <t>% OFF / Desconto Comercial</t>
+  </si>
+  <si>
+    <t>OPCIONAL</t>
+  </si>
+  <si>
+    <t>Percentual (%)</t>
+  </si>
+  <si>
+    <t>Percentual de desconto comercial negociado sobre o pedido (ex: 0%, 5%, 10%). O sistema registra no cabeçalho e preserva os preços unitários líquidos da grade.</t>
+  </si>
+  <si>
+    <t>% NOTA FISCAL</t>
+  </si>
+  <si>
+    <t>Percentual do valor faturado oficialmente em Nota Fiscal (padrão: 100%). Usado para controle fiscal e histórico.</t>
+  </si>
+  <si>
     <t>Texto ou Número</t>
   </si>
   <si>
     <t>Referência do item de acordo com a tabela do fornecedor (ex: 652, REF-1020).</t>
   </si>
   <si>
-    <t>OPCIONAL</t>
-  </si>
-  <si>
     <t>PRD-XXXX</t>
   </si>
   <si>
@@ -532,16 +529,7 @@
     <t>Moeda (R$)</t>
   </si>
   <si>
-    <t>Preço unitário líquido de compra da peça já com descontos comerciais aplicados.</t>
-  </si>
-  <si>
-    <t>Percentual (%)</t>
-  </si>
-  <si>
-    <t>Alíquota de IPI se houver incidência.</t>
-  </si>
-  <si>
-    <t>Preço pretendido de venda ao consumidor final na gôndola das 20 lojas da Rede Mega 12.</t>
+    <t>Preço unitário líquido de compra da peça negociado com o fornecedor.</t>
   </si>
   <si>
     <t>Aba SEPARAÇÃO POR LOJA</t>
@@ -620,11 +608,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -641,7 +628,7 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -737,16 +724,6 @@
       <name val="Segoe UI"/>
     </font>
     <font>
-      <color rgb="FF0F172A"/>
-      <sz val="8.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <color rgb="FF92400E"/>
-      <sz val="8.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
       <color rgb="FF059669"/>
       <sz val="8.5"/>
       <name val="Segoe UI"/>
@@ -764,31 +741,8 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF064E3B"/>
-      <sz val="8.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF064E3B"/>
-      <sz val="9.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF991B1B"/>
       <sz val="8.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <color rgb="FF475569"/>
-      <sz val="8"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -876,7 +830,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -961,21 +915,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF064E3B"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF064E3B"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF064E3B"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF064E3B"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFEF4444"/>
       </left>
       <right style="thin">
@@ -983,19 +922,6 @@
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF064E3B"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF064E3B"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF064E3B"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1015,7 +941,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1087,24 +1013,9 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="15" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1120,97 +1031,43 @@
     <xf numFmtId="0" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="15" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="23" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1234,19 +1091,19 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1278,7 +1135,7 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1620,25 +1477,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="4" width="18" customWidth="1"/>
+    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="44" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
-    <col min="16" max="16" width="15" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1649,18 +1502,13 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-    </row>
-    <row r="2" ht="18" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -1671,18 +1519,13 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -1696,14 +1539,9 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
@@ -1711,21 +1549,16 @@
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="F5" s="6" t="s">
+        <v>6</v>
+      </c>
       <c r="G5" s="6"/>
-      <c r="H5" s="6" t="s">
-        <v>6</v>
-      </c>
+      <c r="H5" s="6"/>
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-    </row>
-    <row r="6" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
@@ -1735,23 +1568,18 @@
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="G6" s="10" t="s">
         <v>9</v>
       </c>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-    </row>
-    <row r="7" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
@@ -1761,23 +1589,18 @@
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
       <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="G7" s="10" t="s">
         <v>13</v>
       </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-    </row>
-    <row r="8" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -1787,23 +1610,18 @@
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="G8" s="10" t="s">
         <v>17</v>
       </c>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-    </row>
-    <row r="9" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>18</v>
       </c>
@@ -1813,23 +1631,18 @@
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="G9" s="10" t="s">
         <v>21</v>
       </c>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-    </row>
-    <row r="10" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
@@ -1839,24 +1652,19 @@
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="9" t="s">
+      <c r="F10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="G10" s="10" t="s">
         <v>25</v>
       </c>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
     </row>
     <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>26</v>
       </c>
@@ -1870,82 +1678,67 @@
       <c r="I12" s="12"/>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-    </row>
-    <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>27</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="13" t="s">
+      <c r="C13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="D13" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="14"/>
+      <c r="E13" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="G13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I13" s="14"/>
-      <c r="J13" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="K13" s="15" t="s">
+      <c r="H13" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="13" t="s">
+      <c r="I13" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="M13" s="14" t="s">
+      <c r="J13" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="N13" s="14"/>
-      <c r="O13" s="13" t="s">
+      <c r="K13" s="14"/>
+    </row>
+    <row r="14" ht="19" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="P13" s="15" t="s">
+      <c r="B14" s="15" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="C14" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="D14" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="13" t="s">
+      <c r="E14" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="F14" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="F14" s="16"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
       <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="16"/>
     </row>
     <row r="15" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="25" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" ht="25" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>43</v>
       </c>
@@ -1979,43 +1772,28 @@
       <c r="K16" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="M16" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="N16" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="O16" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="P16" s="19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="20">
         <v>1</v>
       </c>
       <c r="B17" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="23" t="s">
         <v>59</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="F17" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>64</v>
       </c>
       <c r="H17" s="23">
         <v>6</v>
@@ -2030,100 +1808,64 @@
       <c r="K17" s="25">
         <v>4.7</v>
       </c>
-      <c r="L17" s="26">
-        <v>0.05</v>
-      </c>
-      <c r="M17" s="27">
-        <f>J17*K17*L17</f>
-        <v>28.200000000000003</v>
-      </c>
-      <c r="N17" s="28">
-        <f>J17*K17</f>
-        <v>564</v>
-      </c>
-      <c r="O17" s="29">
-        <v>12</v>
-      </c>
-      <c r="P17" s="30">
-        <f>IF(O17&gt;0,(O17-K17)/O17,0)</f>
-        <v>0.6083333333333333</v>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="31">
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="26">
         <v>2</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>68</v>
-      </c>
-      <c r="F18" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="G18" s="34" t="s">
+      <c r="B18" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="F18" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="H18" s="34">
+      <c r="G18" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18" s="29">
         <v>6</v>
       </c>
-      <c r="I18" s="32">
+      <c r="I18" s="27">
         <v>15</v>
       </c>
-      <c r="J18" s="33">
+      <c r="J18" s="28">
         <f>H18*I18</f>
         <v>90</v>
       </c>
-      <c r="K18" s="36">
+      <c r="K18" s="31">
         <v>6.5</v>
       </c>
-      <c r="L18" s="37">
-        <v>0</v>
-      </c>
-      <c r="M18" s="38">
-        <f>J18*K18*L18</f>
-        <v>0</v>
-      </c>
-      <c r="N18" s="39">
-        <f>J18*K18</f>
-        <v>585</v>
-      </c>
-      <c r="O18" s="40">
-        <v>15</v>
-      </c>
-      <c r="P18" s="41">
-        <f>IF(O18&gt;0,(O18-K18)/O18,0)</f>
-        <v>0.5666666666666667</v>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="20">
         <v>3</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H19" s="23">
         <v>6</v>
@@ -2138,100 +1880,64 @@
       <c r="K19" s="25">
         <v>6.5</v>
       </c>
-      <c r="L19" s="26">
-        <v>0</v>
-      </c>
-      <c r="M19" s="42">
-        <f>J19*K19*L19</f>
-        <v>0</v>
-      </c>
-      <c r="N19" s="28">
-        <f>J19*K19</f>
-        <v>468</v>
-      </c>
-      <c r="O19" s="29">
-        <v>15</v>
-      </c>
-      <c r="P19" s="30">
-        <f>IF(O19&gt;0,(O19-K19)/O19,0)</f>
-        <v>0.5666666666666667</v>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="31">
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="26">
         <v>4</v>
       </c>
-      <c r="B20" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="D20" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F20" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="G20" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="H20" s="34">
+      <c r="B20" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="E20" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="H20" s="29">
         <v>6</v>
       </c>
-      <c r="I20" s="32">
+      <c r="I20" s="27">
         <v>18</v>
       </c>
-      <c r="J20" s="33">
+      <c r="J20" s="28">
         <f>H20*I20</f>
         <v>108</v>
       </c>
-      <c r="K20" s="36">
+      <c r="K20" s="31">
         <v>7.4</v>
       </c>
-      <c r="L20" s="37">
-        <v>0.08</v>
-      </c>
-      <c r="M20" s="43">
-        <f>J20*K20*L20</f>
-        <v>63.93600000000001</v>
-      </c>
-      <c r="N20" s="39">
-        <f>J20*K20</f>
-        <v>799.2</v>
-      </c>
-      <c r="O20" s="40">
-        <v>19.9</v>
-      </c>
-      <c r="P20" s="41">
-        <f>IF(O20&gt;0,(O20-K20)/O20,0)</f>
-        <v>0.6281407035175879</v>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="20">
         <v>5</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="C21" s="44" t="s">
-        <v>80</v>
+        <v>74</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>75</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H21" s="23">
         <v>12</v>
@@ -2246,787 +1952,480 @@
       <c r="K21" s="25">
         <v>6.2</v>
       </c>
-      <c r="L21" s="26">
-        <v>0</v>
-      </c>
-      <c r="M21" s="42">
-        <f>J21*K21*L21</f>
-        <v>0</v>
-      </c>
-      <c r="N21" s="28">
-        <f>J21*K21</f>
-        <v>744</v>
-      </c>
-      <c r="O21" s="29">
-        <v>12</v>
-      </c>
-      <c r="P21" s="30">
-        <f>IF(O21&gt;0,(O21-K21)/O21,0)</f>
-        <v>0.48333333333333334</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="45">
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="33">
         <v>6</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H22" s="45">
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H22" s="33">
         <v>1</v>
       </c>
-      <c r="I22" s="46"/>
-      <c r="J22" s="45">
+      <c r="I22" s="34"/>
+      <c r="J22" s="33">
         <f>IF(I22&gt;0,H22*I22,0)</f>
         <v>0</v>
       </c>
-      <c r="K22" s="47"/>
-      <c r="L22" s="48">
-        <v>0</v>
-      </c>
-      <c r="M22" s="47">
-        <f>IF(L22&gt;0,J22*K22*L22,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N22" s="47">
-        <f>IF(J22&gt;0,J22*K22,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O22" s="47"/>
-      <c r="P22" s="49">
-        <f>IF(O22&gt;0,(O22-K22)/O22,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="50">
+      <c r="K22" s="35"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="36">
         <v>7</v>
       </c>
-      <c r="B23" s="51"/>
-      <c r="C23" s="51"/>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="51"/>
-      <c r="G23" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H23" s="50">
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H23" s="36">
         <v>1</v>
       </c>
-      <c r="I23" s="51"/>
-      <c r="J23" s="50">
+      <c r="I23" s="37"/>
+      <c r="J23" s="36">
         <f>IF(I23&gt;0,H23*I23,0)</f>
         <v>0</v>
       </c>
-      <c r="K23" s="52"/>
-      <c r="L23" s="53">
-        <v>0</v>
-      </c>
-      <c r="M23" s="52">
-        <f>IF(L23&gt;0,J23*K23*L23,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N23" s="52">
-        <f>IF(J23&gt;0,J23*K23,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O23" s="52"/>
-      <c r="P23" s="54">
-        <f>IF(O23&gt;0,(O23-K23)/O23,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="45">
+      <c r="K23" s="38"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="33">
         <v>8</v>
       </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H24" s="45">
+      <c r="B24" s="34"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H24" s="33">
         <v>1</v>
       </c>
-      <c r="I24" s="46"/>
-      <c r="J24" s="45">
+      <c r="I24" s="34"/>
+      <c r="J24" s="33">
         <f>IF(I24&gt;0,H24*I24,0)</f>
         <v>0</v>
       </c>
-      <c r="K24" s="47"/>
-      <c r="L24" s="48">
-        <v>0</v>
-      </c>
-      <c r="M24" s="47">
-        <f>IF(L24&gt;0,J24*K24*L24,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N24" s="47">
-        <f>IF(J24&gt;0,J24*K24,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O24" s="47"/>
-      <c r="P24" s="49">
-        <f>IF(O24&gt;0,(O24-K24)/O24,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="50">
+      <c r="K24" s="35"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="36">
         <v>9</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H25" s="50">
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H25" s="36">
         <v>1</v>
       </c>
-      <c r="I25" s="51"/>
-      <c r="J25" s="50">
+      <c r="I25" s="37"/>
+      <c r="J25" s="36">
         <f>IF(I25&gt;0,H25*I25,0)</f>
         <v>0</v>
       </c>
-      <c r="K25" s="52"/>
-      <c r="L25" s="53">
-        <v>0</v>
-      </c>
-      <c r="M25" s="52">
-        <f>IF(L25&gt;0,J25*K25*L25,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="52">
-        <f>IF(J25&gt;0,J25*K25,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O25" s="52"/>
-      <c r="P25" s="54">
-        <f>IF(O25&gt;0,(O25-K25)/O25,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="45">
+      <c r="K25" s="38"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="33">
         <v>10</v>
       </c>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H26" s="45">
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H26" s="33">
         <v>1</v>
       </c>
-      <c r="I26" s="46"/>
-      <c r="J26" s="45">
+      <c r="I26" s="34"/>
+      <c r="J26" s="33">
         <f>IF(I26&gt;0,H26*I26,0)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="47"/>
-      <c r="L26" s="48">
-        <v>0</v>
-      </c>
-      <c r="M26" s="47">
-        <f>IF(L26&gt;0,J26*K26*L26,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N26" s="47">
-        <f>IF(J26&gt;0,J26*K26,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O26" s="47"/>
-      <c r="P26" s="49">
-        <f>IF(O26&gt;0,(O26-K26)/O26,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="50">
+      <c r="K26" s="35"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="36">
         <v>11</v>
       </c>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H27" s="50">
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H27" s="36">
         <v>1</v>
       </c>
-      <c r="I27" s="51"/>
-      <c r="J27" s="50">
+      <c r="I27" s="37"/>
+      <c r="J27" s="36">
         <f>IF(I27&gt;0,H27*I27,0)</f>
         <v>0</v>
       </c>
-      <c r="K27" s="52"/>
-      <c r="L27" s="53">
-        <v>0</v>
-      </c>
-      <c r="M27" s="52">
-        <f>IF(L27&gt;0,J27*K27*L27,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N27" s="52">
-        <f>IF(J27&gt;0,J27*K27,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O27" s="52"/>
-      <c r="P27" s="54">
-        <f>IF(O27&gt;0,(O27-K27)/O27,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="45">
+      <c r="K27" s="38"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="33">
         <v>12</v>
       </c>
-      <c r="B28" s="46"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H28" s="45">
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H28" s="33">
         <v>1</v>
       </c>
-      <c r="I28" s="46"/>
-      <c r="J28" s="45">
+      <c r="I28" s="34"/>
+      <c r="J28" s="33">
         <f>IF(I28&gt;0,H28*I28,0)</f>
         <v>0</v>
       </c>
-      <c r="K28" s="47"/>
-      <c r="L28" s="48">
-        <v>0</v>
-      </c>
-      <c r="M28" s="47">
-        <f>IF(L28&gt;0,J28*K28*L28,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N28" s="47">
-        <f>IF(J28&gt;0,J28*K28,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O28" s="47"/>
-      <c r="P28" s="49">
-        <f>IF(O28&gt;0,(O28-K28)/O28,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="50">
+      <c r="K28" s="35"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="36">
         <v>13</v>
       </c>
-      <c r="B29" s="51"/>
-      <c r="C29" s="51"/>
-      <c r="D29" s="51"/>
-      <c r="E29" s="51"/>
-      <c r="F29" s="51"/>
-      <c r="G29" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H29" s="50">
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H29" s="36">
         <v>1</v>
       </c>
-      <c r="I29" s="51"/>
-      <c r="J29" s="50">
+      <c r="I29" s="37"/>
+      <c r="J29" s="36">
         <f>IF(I29&gt;0,H29*I29,0)</f>
         <v>0</v>
       </c>
-      <c r="K29" s="52"/>
-      <c r="L29" s="53">
-        <v>0</v>
-      </c>
-      <c r="M29" s="52">
-        <f>IF(L29&gt;0,J29*K29*L29,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N29" s="52">
-        <f>IF(J29&gt;0,J29*K29,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O29" s="52"/>
-      <c r="P29" s="54">
-        <f>IF(O29&gt;0,(O29-K29)/O29,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="45">
+      <c r="K29" s="38"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="33">
         <v>14</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H30" s="45">
+      <c r="B30" s="34"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H30" s="33">
         <v>1</v>
       </c>
-      <c r="I30" s="46"/>
-      <c r="J30" s="45">
+      <c r="I30" s="34"/>
+      <c r="J30" s="33">
         <f>IF(I30&gt;0,H30*I30,0)</f>
         <v>0</v>
       </c>
-      <c r="K30" s="47"/>
-      <c r="L30" s="48">
-        <v>0</v>
-      </c>
-      <c r="M30" s="47">
-        <f>IF(L30&gt;0,J30*K30*L30,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N30" s="47">
-        <f>IF(J30&gt;0,J30*K30,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O30" s="47"/>
-      <c r="P30" s="49">
-        <f>IF(O30&gt;0,(O30-K30)/O30,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="50">
+      <c r="K30" s="35"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="36">
         <v>15</v>
       </c>
-      <c r="B31" s="51"/>
-      <c r="C31" s="51"/>
-      <c r="D31" s="51"/>
-      <c r="E31" s="51"/>
-      <c r="F31" s="51"/>
-      <c r="G31" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H31" s="50">
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H31" s="36">
         <v>1</v>
       </c>
-      <c r="I31" s="51"/>
-      <c r="J31" s="50">
+      <c r="I31" s="37"/>
+      <c r="J31" s="36">
         <f>IF(I31&gt;0,H31*I31,0)</f>
         <v>0</v>
       </c>
-      <c r="K31" s="52"/>
-      <c r="L31" s="53">
-        <v>0</v>
-      </c>
-      <c r="M31" s="52">
-        <f>IF(L31&gt;0,J31*K31*L31,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N31" s="52">
-        <f>IF(J31&gt;0,J31*K31,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O31" s="52"/>
-      <c r="P31" s="54">
-        <f>IF(O31&gt;0,(O31-K31)/O31,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="45">
+      <c r="K31" s="38"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="33">
         <v>16</v>
       </c>
-      <c r="B32" s="46"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="46"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H32" s="45">
+      <c r="B32" s="34"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H32" s="33">
         <v>1</v>
       </c>
-      <c r="I32" s="46"/>
-      <c r="J32" s="45">
+      <c r="I32" s="34"/>
+      <c r="J32" s="33">
         <f>IF(I32&gt;0,H32*I32,0)</f>
         <v>0</v>
       </c>
-      <c r="K32" s="47"/>
-      <c r="L32" s="48">
-        <v>0</v>
-      </c>
-      <c r="M32" s="47">
-        <f>IF(L32&gt;0,J32*K32*L32,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N32" s="47">
-        <f>IF(J32&gt;0,J32*K32,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O32" s="47"/>
-      <c r="P32" s="49">
-        <f>IF(O32&gt;0,(O32-K32)/O32,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="50">
+      <c r="K32" s="35"/>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="36">
         <v>17</v>
       </c>
-      <c r="B33" s="51"/>
-      <c r="C33" s="51"/>
-      <c r="D33" s="51"/>
-      <c r="E33" s="51"/>
-      <c r="F33" s="51"/>
-      <c r="G33" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H33" s="50">
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H33" s="36">
         <v>1</v>
       </c>
-      <c r="I33" s="51"/>
-      <c r="J33" s="50">
+      <c r="I33" s="37"/>
+      <c r="J33" s="36">
         <f>IF(I33&gt;0,H33*I33,0)</f>
         <v>0</v>
       </c>
-      <c r="K33" s="52"/>
-      <c r="L33" s="53">
-        <v>0</v>
-      </c>
-      <c r="M33" s="52">
-        <f>IF(L33&gt;0,J33*K33*L33,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N33" s="52">
-        <f>IF(J33&gt;0,J33*K33,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O33" s="52"/>
-      <c r="P33" s="54">
-        <f>IF(O33&gt;0,(O33-K33)/O33,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="45">
+      <c r="K33" s="38"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="33">
         <v>18</v>
       </c>
-      <c r="B34" s="46"/>
-      <c r="C34" s="46"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="46"/>
-      <c r="F34" s="46"/>
-      <c r="G34" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H34" s="45">
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H34" s="33">
         <v>1</v>
       </c>
-      <c r="I34" s="46"/>
-      <c r="J34" s="45">
+      <c r="I34" s="34"/>
+      <c r="J34" s="33">
         <f>IF(I34&gt;0,H34*I34,0)</f>
         <v>0</v>
       </c>
-      <c r="K34" s="47"/>
-      <c r="L34" s="48">
-        <v>0</v>
-      </c>
-      <c r="M34" s="47">
-        <f>IF(L34&gt;0,J34*K34*L34,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N34" s="47">
-        <f>IF(J34&gt;0,J34*K34,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O34" s="47"/>
-      <c r="P34" s="49">
-        <f>IF(O34&gt;0,(O34-K34)/O34,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A35" s="50">
+      <c r="K34" s="35"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="36">
         <v>19</v>
       </c>
-      <c r="B35" s="51"/>
-      <c r="C35" s="51"/>
-      <c r="D35" s="51"/>
-      <c r="E35" s="51"/>
-      <c r="F35" s="51"/>
-      <c r="G35" s="50" t="s">
-        <v>84</v>
-      </c>
-      <c r="H35" s="50">
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H35" s="36">
         <v>1</v>
       </c>
-      <c r="I35" s="51"/>
-      <c r="J35" s="50">
+      <c r="I35" s="37"/>
+      <c r="J35" s="36">
         <f>IF(I35&gt;0,H35*I35,0)</f>
         <v>0</v>
       </c>
-      <c r="K35" s="52"/>
-      <c r="L35" s="53">
-        <v>0</v>
-      </c>
-      <c r="M35" s="52">
-        <f>IF(L35&gt;0,J35*K35*L35,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N35" s="52">
-        <f>IF(J35&gt;0,J35*K35,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O35" s="52"/>
-      <c r="P35" s="54">
-        <f>IF(O35&gt;0,(O35-K35)/O35,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A36" s="45">
+      <c r="K35" s="38"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="33">
         <v>20</v>
       </c>
-      <c r="B36" s="46"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="46"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H36" s="45">
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="H36" s="33">
         <v>1</v>
       </c>
-      <c r="I36" s="46"/>
-      <c r="J36" s="45">
+      <c r="I36" s="34"/>
+      <c r="J36" s="33">
         <f>IF(I36&gt;0,H36*I36,0)</f>
         <v>0</v>
       </c>
-      <c r="K36" s="47"/>
-      <c r="L36" s="48">
-        <v>0</v>
-      </c>
-      <c r="M36" s="47">
-        <f>IF(L36&gt;0,J36*K36*L36,0)</f>
-        <v>0</v>
-      </c>
-      <c r="N36" s="47">
-        <f>IF(J36&gt;0,J36*K36,0)</f>
-        <v>0</v>
-      </c>
-      <c r="O36" s="47"/>
-      <c r="P36" s="49">
-        <f>IF(O36&gt;0,(O36-K36)/O36,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" s="55" t="s">
-        <v>85</v>
-      </c>
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="55"/>
-      <c r="H37" s="55"/>
-      <c r="I37" s="56">
+      <c r="K36" s="35"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" s="39"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="40">
         <f>SUM(I17:I36)</f>
         <v>75</v>
       </c>
-      <c r="J37" s="56">
+      <c r="J37" s="40">
         <f>SUM(J17:J36)</f>
         <v>516</v>
       </c>
-      <c r="K37" s="57">
-        <f>IF(J37&gt;0,N37/J37,0)</f>
-        <v>6.09</v>
-      </c>
-      <c r="L37" s="58" t="s">
-        <v>80</v>
-      </c>
-      <c r="M37" s="59">
-        <f>SUM(M17:M36)</f>
-        <v>92.42</v>
-      </c>
-      <c r="N37" s="60">
-        <f>SUM(N17:N36)</f>
-        <v>3144.6</v>
-      </c>
-      <c r="O37" s="57">
-        <f>AVERAGE(O17:O21)</f>
-        <v>14.78</v>
-      </c>
-      <c r="P37" s="61">
-        <f>IF(O37&gt;0,(O37-K37)/O37,0)</f>
-        <v>0.588</v>
+      <c r="K37" s="41" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="38" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A39" s="62" t="s">
+    <row r="39" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" s="42"/>
+      <c r="C39" s="42"/>
+      <c r="D39" s="42"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="42"/>
+      <c r="G39" s="42"/>
+      <c r="H39" s="42"/>
+      <c r="I39" s="42"/>
+      <c r="J39" s="42"/>
+      <c r="K39" s="42"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="43"/>
+      <c r="I40" s="43"/>
+      <c r="J40" s="43"/>
+      <c r="K40" s="43"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" s="43"/>
+      <c r="C41" s="43"/>
+      <c r="D41" s="43"/>
+      <c r="E41" s="43"/>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+      <c r="H41" s="43"/>
+      <c r="I41" s="43"/>
+      <c r="J41" s="43"/>
+      <c r="K41" s="43"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" s="43"/>
+      <c r="C42" s="43"/>
+      <c r="D42" s="43"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="43"/>
+      <c r="G42" s="43"/>
+      <c r="H42" s="43"/>
+      <c r="I42" s="43"/>
+      <c r="J42" s="43"/>
+      <c r="K42" s="43"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" s="43"/>
+      <c r="C43" s="43"/>
+      <c r="D43" s="43"/>
+      <c r="E43" s="43"/>
+      <c r="F43" s="43"/>
+      <c r="G43" s="43"/>
+      <c r="H43" s="43"/>
+      <c r="I43" s="43"/>
+      <c r="J43" s="43"/>
+      <c r="K43" s="43"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="B39" s="62"/>
-      <c r="C39" s="62"/>
-      <c r="D39" s="62"/>
-      <c r="E39" s="62"/>
-      <c r="F39" s="62"/>
-      <c r="G39" s="62"/>
-      <c r="H39" s="62"/>
-      <c r="I39" s="62"/>
-      <c r="J39" s="62"/>
-      <c r="L39" s="63" t="s">
-        <v>87</v>
-      </c>
-      <c r="M39" s="63"/>
-      <c r="N39" s="63"/>
-      <c r="O39" s="63"/>
-      <c r="P39" s="63"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="64" t="s">
-        <v>88</v>
-      </c>
-      <c r="B40" s="64"/>
-      <c r="C40" s="64"/>
-      <c r="D40" s="64"/>
-      <c r="E40" s="64"/>
-      <c r="F40" s="64"/>
-      <c r="G40" s="64"/>
-      <c r="H40" s="64"/>
-      <c r="I40" s="64"/>
-      <c r="J40" s="64"/>
-      <c r="L40" s="65">
-        <f>N37+M37</f>
-        <v>3237.02</v>
-      </c>
-      <c r="M40" s="65"/>
-      <c r="N40" s="65"/>
-      <c r="O40" s="65"/>
-      <c r="P40" s="65"/>
-    </row>
-    <row r="41" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A41" s="64" t="s">
-        <v>89</v>
-      </c>
-      <c r="B41" s="64"/>
-      <c r="C41" s="64"/>
-      <c r="D41" s="64"/>
-      <c r="E41" s="64"/>
-      <c r="F41" s="64"/>
-      <c r="G41" s="64"/>
-      <c r="H41" s="64"/>
-      <c r="I41" s="64"/>
-      <c r="J41" s="64"/>
-      <c r="L41" s="65"/>
-      <c r="M41" s="65"/>
-      <c r="N41" s="65"/>
-      <c r="O41" s="65"/>
-      <c r="P41" s="65"/>
-    </row>
-    <row r="42" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="64" t="s">
-        <v>90</v>
-      </c>
-      <c r="B42" s="64"/>
-      <c r="C42" s="64"/>
-      <c r="D42" s="64"/>
-      <c r="E42" s="64"/>
-      <c r="F42" s="64"/>
-      <c r="G42" s="64"/>
-      <c r="H42" s="64"/>
-      <c r="I42" s="64"/>
-      <c r="J42" s="64"/>
-      <c r="L42" s="66" t="str">
-        <f>="Líquido: " &amp; TEXT(N37,"R$ #,##0.00") &amp; " | IPI: " &amp; TEXT(M37,"R$ #,##0.00")</f>
-        <v>Líquido: R$ 3.144,60 | IPI: R$ 92,42</v>
-      </c>
-      <c r="M42" s="66"/>
-      <c r="N42" s="66"/>
-      <c r="O42" s="66"/>
-      <c r="P42" s="66"/>
-    </row>
-    <row r="43" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="64" t="s">
-        <v>91</v>
-      </c>
-      <c r="B43" s="64"/>
-      <c r="C43" s="64"/>
-      <c r="D43" s="64"/>
-      <c r="E43" s="64"/>
-      <c r="F43" s="64"/>
-      <c r="G43" s="64"/>
-      <c r="H43" s="64"/>
-      <c r="I43" s="64"/>
-      <c r="J43" s="64"/>
-    </row>
-    <row r="44" ht="17" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="67" t="s">
-        <v>92</v>
-      </c>
-      <c r="B44" s="67"/>
-      <c r="C44" s="67"/>
-      <c r="D44" s="67"/>
-      <c r="E44" s="67"/>
-      <c r="F44" s="67"/>
-      <c r="G44" s="67"/>
-      <c r="H44" s="67"/>
-      <c r="I44" s="67"/>
-      <c r="J44" s="67"/>
+      <c r="B44" s="44"/>
+      <c r="C44" s="44"/>
+      <c r="D44" s="44"/>
+      <c r="E44" s="44"/>
+      <c r="F44" s="44"/>
+      <c r="G44" s="44"/>
+      <c r="H44" s="44"/>
+      <c r="I44" s="44"/>
+      <c r="J44" s="44"/>
+      <c r="K44" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="L1:P1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="L2:P2"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="H5:P5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="I6:P6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="I7:P7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="I8:P8"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="I9:P9"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="I10:P10"/>
-    <mergeCell ref="A12:P12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E14:P14"/>
+  <mergeCells count="27">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="F5:K5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="G10:K10"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="F14:K14"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A39:J39"/>
-    <mergeCell ref="L39:P39"/>
-    <mergeCell ref="A40:J40"/>
-    <mergeCell ref="L40:P41"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="A42:J42"/>
-    <mergeCell ref="L42:P42"/>
-    <mergeCell ref="A43:J43"/>
-    <mergeCell ref="A44:J44"/>
+    <mergeCell ref="A39:K39"/>
+    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="A44:K44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3050,7 +2449,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3082,179 +2481,179 @@
       <c r="AC1" s="1"/>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="45" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="45"/>
+      <c r="X2" s="45"/>
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
+      <c r="AB2" s="45"/>
+      <c r="AC2" s="45"/>
+    </row>
+    <row r="3" ht="18" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="47" t="s">
+        <v>90</v>
+      </c>
+      <c r="G3" s="48" t="s">
+        <v>91</v>
+      </c>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="P3" s="49"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="49"/>
+      <c r="S3" s="49"/>
+      <c r="T3" s="49"/>
+      <c r="U3" s="49"/>
+      <c r="V3" s="49"/>
+      <c r="W3" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="X3" s="50"/>
+      <c r="Y3" s="50"/>
+      <c r="Z3" s="50"/>
+      <c r="AA3" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="68"/>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
-      <c r="U2" s="68"/>
-      <c r="V2" s="68"/>
-      <c r="W2" s="68"/>
-      <c r="X2" s="68"/>
-      <c r="Y2" s="68"/>
-      <c r="Z2" s="68"/>
-      <c r="AA2" s="68"/>
-      <c r="AB2" s="68"/>
-      <c r="AC2" s="68"/>
-    </row>
-    <row r="3" ht="18" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A3" s="69" t="s">
+      <c r="AB3" s="46"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A4" s="51" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="70" t="s">
+      <c r="C4" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="G3" s="71" t="s">
+      <c r="D4" s="51" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="51" t="s">
         <v>97</v>
       </c>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
-      <c r="O3" s="72" t="s">
+      <c r="F4" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="P3" s="72"/>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="72"/>
-      <c r="S3" s="72"/>
-      <c r="T3" s="72"/>
-      <c r="U3" s="72"/>
-      <c r="V3" s="72"/>
-      <c r="W3" s="73" t="s">
+      <c r="G4" s="51" t="s">
         <v>99</v>
       </c>
-      <c r="X3" s="73"/>
-      <c r="Y3" s="73"/>
-      <c r="Z3" s="73"/>
-      <c r="AA3" s="69" t="s">
+      <c r="H4" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="AB3" s="69"/>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A4" s="74" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="74" t="s">
+      <c r="I4" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="74" t="s">
+      <c r="J4" s="51" t="s">
         <v>102</v>
       </c>
-      <c r="D4" s="74" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="74" t="s">
+      <c r="K4" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="F4" s="74" t="s">
+      <c r="L4" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="G4" s="74" t="s">
+      <c r="M4" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="H4" s="74" t="s">
+      <c r="N4" s="51" t="s">
         <v>106</v>
       </c>
-      <c r="I4" s="74" t="s">
+      <c r="O4" s="51" t="s">
         <v>107</v>
       </c>
-      <c r="J4" s="74" t="s">
+      <c r="P4" s="51" t="s">
         <v>108</v>
       </c>
-      <c r="K4" s="74" t="s">
+      <c r="Q4" s="51" t="s">
         <v>109</v>
       </c>
-      <c r="L4" s="74" t="s">
+      <c r="R4" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="M4" s="74" t="s">
+      <c r="S4" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="N4" s="74" t="s">
+      <c r="T4" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="O4" s="74" t="s">
+      <c r="U4" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="P4" s="74" t="s">
+      <c r="V4" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="Q4" s="74" t="s">
+      <c r="W4" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="R4" s="74" t="s">
+      <c r="X4" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="S4" s="74" t="s">
+      <c r="Y4" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="T4" s="74" t="s">
+      <c r="Z4" s="51" t="s">
         <v>118</v>
       </c>
-      <c r="U4" s="74" t="s">
+      <c r="AA4" s="51" t="s">
         <v>119</v>
       </c>
-      <c r="V4" s="74" t="s">
+      <c r="AB4" s="51" t="s">
         <v>120</v>
       </c>
-      <c r="W4" s="74" t="s">
-        <v>121</v>
-      </c>
-      <c r="X4" s="74" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y4" s="74" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z4" s="74" t="s">
-        <v>124</v>
-      </c>
-      <c r="AA4" s="74" t="s">
-        <v>125</v>
-      </c>
-      <c r="AB4" s="74" t="s">
-        <v>126</v>
-      </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="75">
+      <c r="A5" s="52">
         <v>1</v>
       </c>
-      <c r="B5" s="76" t="str">
+      <c r="B5" s="53" t="str">
         <f>='PEDIDO COMERCIAL'!B17</f>
         <v>652</v>
       </c>
-      <c r="C5" s="75" t="str">
+      <c r="C5" s="52" t="str">
         <f>='PEDIDO COMERCIAL'!C17</f>
         <v>PRD-001</v>
       </c>
-      <c r="D5" s="77" t="str">
+      <c r="D5" s="54" t="str">
         <f>='PEDIDO COMERCIAL'!E17</f>
         <v>INCENSARIO MOTIVACIONAL EM MADEIRA 25CM</v>
       </c>
@@ -3262,70 +2661,70 @@
         <f>='PEDIDO COMERCIAL'!J17</f>
         <v>120</v>
       </c>
-      <c r="F5" s="75">
+      <c r="F5" s="52">
         <v>12</v>
       </c>
-      <c r="G5" s="75">
+      <c r="G5" s="52">
         <v>7</v>
       </c>
-      <c r="H5" s="75">
+      <c r="H5" s="52">
         <v>7</v>
       </c>
-      <c r="I5" s="75">
+      <c r="I5" s="52">
         <v>7</v>
       </c>
-      <c r="J5" s="75">
+      <c r="J5" s="52">
         <v>7</v>
       </c>
-      <c r="K5" s="75">
+      <c r="K5" s="52">
         <v>7</v>
       </c>
-      <c r="L5" s="75">
+      <c r="L5" s="52">
         <v>7</v>
       </c>
-      <c r="M5" s="75">
+      <c r="M5" s="52">
         <v>7</v>
       </c>
-      <c r="N5" s="75">
+      <c r="N5" s="52">
         <v>7</v>
       </c>
-      <c r="O5" s="75">
+      <c r="O5" s="52">
         <v>5</v>
       </c>
-      <c r="P5" s="75">
+      <c r="P5" s="52">
         <v>5</v>
       </c>
-      <c r="Q5" s="75">
+      <c r="Q5" s="52">
         <v>5</v>
       </c>
-      <c r="R5" s="75">
+      <c r="R5" s="52">
         <v>5</v>
       </c>
-      <c r="S5" s="75">
+      <c r="S5" s="52">
         <v>5</v>
       </c>
-      <c r="T5" s="75">
+      <c r="T5" s="52">
         <v>5</v>
       </c>
-      <c r="U5" s="75">
+      <c r="U5" s="52">
         <v>5</v>
       </c>
-      <c r="V5" s="75">
+      <c r="V5" s="52">
         <v>5</v>
       </c>
-      <c r="W5" s="75">
+      <c r="W5" s="52">
         <v>3</v>
       </c>
-      <c r="X5" s="75">
+      <c r="X5" s="52">
         <v>3</v>
       </c>
-      <c r="Y5" s="75">
+      <c r="Y5" s="52">
         <v>3</v>
       </c>
-      <c r="Z5" s="75">
+      <c r="Z5" s="52">
         <v>3</v>
       </c>
-      <c r="AA5" s="76">
+      <c r="AA5" s="53">
         <f>SUM(F5:Z5)</f>
         <v>120</v>
       </c>
@@ -3335,110 +2734,110 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="78">
+      <c r="A6" s="55">
         <v>2</v>
       </c>
-      <c r="B6" s="79" t="str">
+      <c r="B6" s="56" t="str">
         <f>='PEDIDO COMERCIAL'!B18</f>
         <v>653</v>
       </c>
-      <c r="C6" s="78" t="str">
+      <c r="C6" s="55" t="str">
         <f>='PEDIDO COMERCIAL'!C18</f>
         <v>PRD-002</v>
       </c>
-      <c r="D6" s="80" t="str">
+      <c r="D6" s="57" t="str">
         <f>='PEDIDO COMERCIAL'!E18</f>
         <v>KIT PETISQUEIRA QUADRADA BAMBU COM 3 DIVISORIAS</v>
       </c>
-      <c r="E6" s="33">
+      <c r="E6" s="28">
         <f>='PEDIDO COMERCIAL'!J18</f>
         <v>90</v>
       </c>
-      <c r="F6" s="78">
+      <c r="F6" s="55">
         <v>9</v>
       </c>
-      <c r="G6" s="78">
+      <c r="G6" s="55">
         <v>5</v>
       </c>
-      <c r="H6" s="78">
+      <c r="H6" s="55">
         <v>5</v>
       </c>
-      <c r="I6" s="78">
+      <c r="I6" s="55">
         <v>5</v>
       </c>
-      <c r="J6" s="78">
+      <c r="J6" s="55">
         <v>5</v>
       </c>
-      <c r="K6" s="78">
+      <c r="K6" s="55">
         <v>5</v>
       </c>
-      <c r="L6" s="78">
+      <c r="L6" s="55">
         <v>5</v>
       </c>
-      <c r="M6" s="78">
+      <c r="M6" s="55">
         <v>5</v>
       </c>
-      <c r="N6" s="78">
+      <c r="N6" s="55">
         <v>5</v>
       </c>
-      <c r="O6" s="78">
+      <c r="O6" s="55">
         <v>4</v>
       </c>
-      <c r="P6" s="78">
+      <c r="P6" s="55">
         <v>4</v>
       </c>
-      <c r="Q6" s="78">
+      <c r="Q6" s="55">
         <v>4</v>
       </c>
-      <c r="R6" s="78">
+      <c r="R6" s="55">
         <v>4</v>
       </c>
-      <c r="S6" s="78">
+      <c r="S6" s="55">
         <v>4</v>
       </c>
-      <c r="T6" s="78">
+      <c r="T6" s="55">
         <v>4</v>
       </c>
-      <c r="U6" s="78">
+      <c r="U6" s="55">
         <v>4</v>
       </c>
-      <c r="V6" s="78">
+      <c r="V6" s="55">
         <v>4</v>
       </c>
-      <c r="W6" s="78">
+      <c r="W6" s="55">
         <v>2</v>
       </c>
-      <c r="X6" s="78">
+      <c r="X6" s="55">
         <v>2</v>
       </c>
-      <c r="Y6" s="78">
+      <c r="Y6" s="55">
         <v>2</v>
       </c>
-      <c r="Z6" s="78">
+      <c r="Z6" s="55">
         <v>2</v>
       </c>
-      <c r="AA6" s="79">
+      <c r="AA6" s="56">
         <f>SUM(F6:Z6)</f>
         <v>90</v>
       </c>
-      <c r="AB6" s="33" t="str">
+      <c r="AB6" s="28" t="str">
         <f>IF(AA6=E6,"OK (100%)","DIVERGENTE")</f>
         <v>OK (100%)</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="75">
+      <c r="A7" s="52">
         <v>3</v>
       </c>
-      <c r="B7" s="76" t="str">
+      <c r="B7" s="53" t="str">
         <f>='PEDIDO COMERCIAL'!B19</f>
         <v>654</v>
       </c>
-      <c r="C7" s="75" t="str">
+      <c r="C7" s="52" t="str">
         <f>='PEDIDO COMERCIAL'!C19</f>
         <v>PRD-003</v>
       </c>
-      <c r="D7" s="77" t="str">
+      <c r="D7" s="54" t="str">
         <f>='PEDIDO COMERCIAL'!E19</f>
         <v>KIT PETISQUEIRA RETANGULAR 4 DIVISORIAS</v>
       </c>
@@ -3446,70 +2845,70 @@
         <f>='PEDIDO COMERCIAL'!J19</f>
         <v>72</v>
       </c>
-      <c r="F7" s="75">
+      <c r="F7" s="52">
         <v>7</v>
       </c>
-      <c r="G7" s="75">
+      <c r="G7" s="52">
         <v>4</v>
       </c>
-      <c r="H7" s="75">
+      <c r="H7" s="52">
         <v>4</v>
       </c>
-      <c r="I7" s="75">
+      <c r="I7" s="52">
         <v>4</v>
       </c>
-      <c r="J7" s="75">
+      <c r="J7" s="52">
         <v>4</v>
       </c>
-      <c r="K7" s="75">
+      <c r="K7" s="52">
         <v>4</v>
       </c>
-      <c r="L7" s="75">
+      <c r="L7" s="52">
         <v>4</v>
       </c>
-      <c r="M7" s="75">
+      <c r="M7" s="52">
         <v>4</v>
       </c>
-      <c r="N7" s="75">
+      <c r="N7" s="52">
         <v>4</v>
       </c>
-      <c r="O7" s="75">
+      <c r="O7" s="52">
         <v>3</v>
       </c>
-      <c r="P7" s="75">
+      <c r="P7" s="52">
         <v>3</v>
       </c>
-      <c r="Q7" s="75">
+      <c r="Q7" s="52">
         <v>3</v>
       </c>
-      <c r="R7" s="75">
+      <c r="R7" s="52">
         <v>3</v>
       </c>
-      <c r="S7" s="75">
+      <c r="S7" s="52">
         <v>3</v>
       </c>
-      <c r="T7" s="75">
+      <c r="T7" s="52">
         <v>3</v>
       </c>
-      <c r="U7" s="75">
+      <c r="U7" s="52">
         <v>3</v>
       </c>
-      <c r="V7" s="75">
+      <c r="V7" s="52">
         <v>3</v>
       </c>
-      <c r="W7" s="75">
+      <c r="W7" s="52">
         <v>2</v>
       </c>
-      <c r="X7" s="75">
+      <c r="X7" s="52">
         <v>2</v>
       </c>
-      <c r="Y7" s="75">
+      <c r="Y7" s="52">
         <v>2</v>
       </c>
-      <c r="Z7" s="75">
+      <c r="Z7" s="52">
         <v>2</v>
       </c>
-      <c r="AA7" s="76">
+      <c r="AA7" s="53">
         <f>SUM(F7:Z7)</f>
         <v>72</v>
       </c>
@@ -3519,110 +2918,110 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="78">
+      <c r="A8" s="55">
         <v>4</v>
       </c>
-      <c r="B8" s="79" t="str">
+      <c r="B8" s="56" t="str">
         <f>='PEDIDO COMERCIAL'!B20</f>
         <v>656</v>
       </c>
-      <c r="C8" s="78" t="str">
+      <c r="C8" s="55" t="str">
         <f>='PEDIDO COMERCIAL'!C20</f>
         <v>PRD-004</v>
       </c>
-      <c r="D8" s="80" t="str">
+      <c r="D8" s="57" t="str">
         <f>='PEDIDO COMERCIAL'!E20</f>
         <v>PORTA TEMPERO TABUA GIRATORIA C/ 5 POTES VIDRO</v>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="28">
         <f>='PEDIDO COMERCIAL'!J20</f>
         <v>108</v>
       </c>
-      <c r="F8" s="78">
+      <c r="F8" s="55">
         <v>11</v>
       </c>
-      <c r="G8" s="78">
+      <c r="G8" s="55">
         <v>6</v>
       </c>
-      <c r="H8" s="78">
+      <c r="H8" s="55">
         <v>6</v>
       </c>
-      <c r="I8" s="78">
+      <c r="I8" s="55">
         <v>6</v>
       </c>
-      <c r="J8" s="78">
+      <c r="J8" s="55">
         <v>6</v>
       </c>
-      <c r="K8" s="78">
+      <c r="K8" s="55">
         <v>6</v>
       </c>
-      <c r="L8" s="78">
+      <c r="L8" s="55">
         <v>6</v>
       </c>
-      <c r="M8" s="78">
+      <c r="M8" s="55">
         <v>6</v>
       </c>
-      <c r="N8" s="78">
+      <c r="N8" s="55">
         <v>6</v>
       </c>
-      <c r="O8" s="78">
+      <c r="O8" s="55">
         <v>4</v>
       </c>
-      <c r="P8" s="78">
+      <c r="P8" s="55">
         <v>4</v>
       </c>
-      <c r="Q8" s="78">
+      <c r="Q8" s="55">
         <v>4</v>
       </c>
-      <c r="R8" s="78">
+      <c r="R8" s="55">
         <v>4</v>
       </c>
-      <c r="S8" s="78">
+      <c r="S8" s="55">
         <v>4</v>
       </c>
-      <c r="T8" s="78">
+      <c r="T8" s="55">
         <v>4</v>
       </c>
-      <c r="U8" s="78">
+      <c r="U8" s="55">
         <v>4</v>
       </c>
-      <c r="V8" s="78">
+      <c r="V8" s="55">
         <v>4</v>
       </c>
-      <c r="W8" s="78">
+      <c r="W8" s="55">
         <v>4</v>
       </c>
-      <c r="X8" s="78">
+      <c r="X8" s="55">
         <v>4</v>
       </c>
-      <c r="Y8" s="78">
+      <c r="Y8" s="55">
         <v>4</v>
       </c>
-      <c r="Z8" s="78">
+      <c r="Z8" s="55">
         <v>4</v>
       </c>
-      <c r="AA8" s="79">
+      <c r="AA8" s="56">
         <f>SUM(F8:Z8)</f>
         <v>108</v>
       </c>
-      <c r="AB8" s="33" t="str">
+      <c r="AB8" s="28" t="str">
         <f>IF(AA8=E8,"OK (100%)","DIVERGENTE")</f>
         <v>OK (100%)</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="75">
+      <c r="A9" s="52">
         <v>5</v>
       </c>
-      <c r="B9" s="76" t="str">
+      <c r="B9" s="53" t="str">
         <f>='PEDIDO COMERCIAL'!B21</f>
         <v>657</v>
       </c>
-      <c r="C9" s="75" t="str">
+      <c r="C9" s="52" t="str">
         <f>='PEDIDO COMERCIAL'!C21</f>
         <v/>
       </c>
-      <c r="D9" s="77" t="str">
+      <c r="D9" s="54" t="str">
         <f>='PEDIDO COMERCIAL'!E21</f>
         <v>QUADRO MINHAS COMPRAS MAGNETICO 11X30CM C/ CANETA</v>
       </c>
@@ -3630,70 +3029,70 @@
         <f>='PEDIDO COMERCIAL'!J21</f>
         <v>120</v>
       </c>
-      <c r="F9" s="75">
+      <c r="F9" s="52">
         <v>12</v>
       </c>
-      <c r="G9" s="75">
+      <c r="G9" s="52">
         <v>7</v>
       </c>
-      <c r="H9" s="75">
+      <c r="H9" s="52">
         <v>7</v>
       </c>
-      <c r="I9" s="75">
+      <c r="I9" s="52">
         <v>7</v>
       </c>
-      <c r="J9" s="75">
+      <c r="J9" s="52">
         <v>7</v>
       </c>
-      <c r="K9" s="75">
+      <c r="K9" s="52">
         <v>7</v>
       </c>
-      <c r="L9" s="75">
+      <c r="L9" s="52">
         <v>7</v>
       </c>
-      <c r="M9" s="75">
+      <c r="M9" s="52">
         <v>7</v>
       </c>
-      <c r="N9" s="75">
+      <c r="N9" s="52">
         <v>7</v>
       </c>
-      <c r="O9" s="75">
+      <c r="O9" s="52">
         <v>5</v>
       </c>
-      <c r="P9" s="75">
+      <c r="P9" s="52">
         <v>5</v>
       </c>
-      <c r="Q9" s="75">
+      <c r="Q9" s="52">
         <v>5</v>
       </c>
-      <c r="R9" s="75">
+      <c r="R9" s="52">
         <v>5</v>
       </c>
-      <c r="S9" s="75">
+      <c r="S9" s="52">
         <v>5</v>
       </c>
-      <c r="T9" s="75">
+      <c r="T9" s="52">
         <v>5</v>
       </c>
-      <c r="U9" s="75">
+      <c r="U9" s="52">
         <v>5</v>
       </c>
-      <c r="V9" s="75">
+      <c r="V9" s="52">
         <v>5</v>
       </c>
-      <c r="W9" s="75">
+      <c r="W9" s="52">
         <v>3</v>
       </c>
-      <c r="X9" s="75">
+      <c r="X9" s="52">
         <v>3</v>
       </c>
-      <c r="Y9" s="75">
+      <c r="Y9" s="52">
         <v>3</v>
       </c>
-      <c r="Z9" s="75">
+      <c r="Z9" s="52">
         <v>3</v>
       </c>
-      <c r="AA9" s="76">
+      <c r="AA9" s="53">
         <f>SUM(F9:Z9)</f>
         <v>120</v>
       </c>
@@ -3731,284 +3130,284 @@
   <sheetData>
     <row r="2" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="45" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="58" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="58" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="58" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="58" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="59" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="81" t="s">
+      <c r="D6" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="C5" s="81" t="s">
+      <c r="E6" s="62" t="s">
         <v>130</v>
       </c>
-      <c r="D5" s="81" t="s">
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="63" t="s">
         <v>131</v>
       </c>
-      <c r="E5" s="81" t="s">
+      <c r="C7" s="64" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="82" t="s">
+      <c r="D7" s="65" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="83" t="s">
+      <c r="E7" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="D6" s="84" t="s">
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="59" t="s">
         <v>135</v>
       </c>
-      <c r="E6" s="85" t="s">
+      <c r="C8" s="67" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" s="61" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="86" t="s">
+      <c r="E8" s="62" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="87" t="s">
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="63" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="88" t="s">
+      <c r="C9" s="68" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" s="65" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="89" t="s">
+      <c r="E9" s="66" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="82" t="s">
+    <row r="10" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="C8" s="90" t="s">
-        <v>138</v>
-      </c>
-      <c r="D8" s="84" t="s">
+      <c r="C10" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="D10" s="61" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="85" t="s">
+      <c r="E10" s="62" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="86" t="s">
+    <row r="11" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="63" t="s">
         <v>144</v>
       </c>
-      <c r="C9" s="91" t="s">
-        <v>134</v>
-      </c>
-      <c r="D9" s="88" t="s">
+      <c r="C11" s="64" t="s">
         <v>145</v>
       </c>
-      <c r="E9" s="89" t="s">
+      <c r="D11" s="65" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="82" t="s">
+      <c r="E11" s="66" t="s">
         <v>147</v>
       </c>
-      <c r="C10" s="83" t="s">
-        <v>134</v>
-      </c>
-      <c r="D10" s="84" t="s">
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="59" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="85" t="s">
+      <c r="C12" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>146</v>
+      </c>
+      <c r="E12" s="62" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="86" t="s">
+    <row r="13" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="91" t="s">
-        <v>134</v>
-      </c>
-      <c r="D11" s="88" t="s">
+      <c r="C13" s="68" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="65" t="s">
         <v>150</v>
       </c>
-      <c r="E11" s="89" t="s">
+      <c r="E13" s="66" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="82" t="s">
+    <row r="14" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="90" t="s">
+      <c r="C14" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="D14" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="D12" s="84" t="s">
+      <c r="E14" s="62" t="s">
         <v>153</v>
       </c>
-      <c r="E12" s="85" t="s">
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="63" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="64" t="s">
+        <v>145</v>
+      </c>
+      <c r="D15" s="65" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="86" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="87" t="s">
-        <v>152</v>
-      </c>
-      <c r="D13" s="88" t="s">
+      <c r="E15" s="66" t="s">
         <v>155</v>
       </c>
-      <c r="E13" s="89" t="s">
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="59" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="D16" s="61" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="82" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="83" t="s">
-        <v>134</v>
-      </c>
-      <c r="D14" s="84" t="s">
+      <c r="E16" s="62" t="s">
         <v>157</v>
       </c>
-      <c r="E14" s="85" t="s">
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="63" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="64" t="s">
+        <v>132</v>
+      </c>
+      <c r="D17" s="65" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="86" t="s">
-        <v>48</v>
-      </c>
-      <c r="C15" s="87" t="s">
-        <v>138</v>
-      </c>
-      <c r="D15" s="88" t="s">
+      <c r="E17" s="66" t="s">
         <v>159</v>
       </c>
-      <c r="E15" s="89" t="s">
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="61" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="82" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="83" t="s">
-        <v>134</v>
-      </c>
-      <c r="D16" s="84" t="s">
+      <c r="E18" s="62" t="s">
         <v>161</v>
       </c>
-      <c r="E16" s="85" t="s">
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="63" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="86" t="s">
+      <c r="C19" s="68" t="s">
+        <v>128</v>
+      </c>
+      <c r="D19" s="65" t="s">
         <v>163</v>
       </c>
-      <c r="C17" s="91" t="s">
-        <v>134</v>
-      </c>
-      <c r="D17" s="88" t="s">
+      <c r="E19" s="66" t="s">
         <v>164</v>
       </c>
-      <c r="E17" s="89" t="s">
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="59" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="82" t="s">
+      <c r="C20" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="61" t="s">
+        <v>163</v>
+      </c>
+      <c r="E20" s="62" t="s">
         <v>166</v>
       </c>
-      <c r="C18" s="83" t="s">
-        <v>134</v>
-      </c>
-      <c r="D18" s="84" t="s">
-        <v>164</v>
-      </c>
-      <c r="E18" s="85" t="s">
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="63" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="69" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="86" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="92" t="s">
+      <c r="D21" s="65" t="s">
         <v>168</v>
       </c>
-      <c r="D19" s="88" t="s">
+      <c r="E21" s="66" t="s">
         <v>169</v>
       </c>
-      <c r="E19" s="89" t="s">
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="59" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="60" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" s="61" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20" s="82" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" s="83" t="s">
-        <v>134</v>
-      </c>
-      <c r="D20" s="84" t="s">
+      <c r="E22" s="62" t="s">
         <v>171</v>
       </c>
-      <c r="E20" s="85" t="s">
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="63" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="86" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="87" t="s">
-        <v>152</v>
-      </c>
-      <c r="D21" s="88" t="s">
+      <c r="C23" s="64" t="s">
+        <v>145</v>
+      </c>
+      <c r="D23" s="65" t="s">
         <v>173</v>
       </c>
-      <c r="E21" s="89" t="s">
+      <c r="E23" s="66" t="s">
         <v>174</v>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="82" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="90" t="s">
-        <v>138</v>
-      </c>
-      <c r="D22" s="84" t="s">
-        <v>171</v>
-      </c>
-      <c r="E22" s="85" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B23" s="86" t="s">
-        <v>176</v>
-      </c>
-      <c r="C23" s="87" t="s">
-        <v>152</v>
-      </c>
-      <c r="D23" s="88" t="s">
-        <v>177</v>
-      </c>
-      <c r="E23" s="89" t="s">
-        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -4034,86 +3433,86 @@
   <sheetData>
     <row r="2" ht="24" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
     <row r="4" ht="22" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="81" t="s">
+      <c r="B4" s="58" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="58" t="s">
+        <v>177</v>
+      </c>
+      <c r="D4" s="58" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="22" t="s">
         <v>180</v>
       </c>
-      <c r="C4" s="81" t="s">
+      <c r="D5" s="62" t="s">
         <v>181</v>
       </c>
-      <c r="D4" s="81" t="s">
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="63" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="82" t="s">
+      <c r="C6" s="28" t="s">
         <v>183</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="D6" s="66" t="s">
         <v>184</v>
       </c>
-      <c r="D5" s="85" t="s">
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="59" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="86" t="s">
+      <c r="C7" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="D7" s="62" t="s">
         <v>187</v>
       </c>
-      <c r="D6" s="89" t="s">
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="63" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="82" t="s">
+      <c r="C8" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="D8" s="66" t="s">
         <v>190</v>
       </c>
-      <c r="D7" s="85" t="s">
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="59" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="86" t="s">
+      <c r="C9" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="D9" s="62" t="s">
         <v>193</v>
       </c>
-      <c r="D8" s="89" t="s">
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="63" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="82" t="s">
+      <c r="C10" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="66" t="s">
         <v>195</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>196</v>
-      </c>
-      <c r="D9" s="85" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="86" t="s">
-        <v>198</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>196</v>
-      </c>
-      <c r="D10" s="89" t="s">
-        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>